<commit_message>
Tracker v2: direct apply links, honest odds column, windows aligned to Apr-2027 start
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MKudDRnoWxq3Vy24DBvgME
</commit_message>
<xml_diff>
--- a/Sponsored-International-Internships.xlsx
+++ b/Sponsored-International-Internships.xlsx
@@ -115,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -130,7 +130,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -139,8 +145,14 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -511,174 +523,123 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SPONSORED INTERNATIONAL INTERNSHIPS &amp; FUNDED PROGRAMS — RYAN EBENEZER G</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="45" customHeight="1">
+          <t>SPONSORED INTERNATIONAL INTERNSHIPS &amp; FUNDED PROGRAMS — RYAN EBENEZER G (v2, 10 Jul 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built 10 Jul 2026. Profile: final year (grad Apr 2027), CGPA 2.8/4.0, founder of Pack &amp; Pass, marketer, non-coder. Priority: 1 = apply this cycle · 2 = opportunistic · 3 = later fork · X = don't waste time (honest skip). Verify every deadline on the official link before applying — windows shift yearly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+          <t>YOUR TIMING: you are only free for a full-time internship from APRIL 2027 (after graduation). The 'When to apply' column is aligned to that. IMPORTANT: competitions &amp; short programs (Red Bull, Brandstorm, Westerwelle, SUSI, P&amp;G, Hult) are days-to-weeks EVENTS — you can do those while still studying; don't wait for April. Only the true internships (KPMG, Big-4, UNICEF, ILO, AIESEC) need your April availability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>YOUR ODDS, honestly: each sponsored program alone is a low-probability bet — that is normal, everyone's odds are low, and your founder profile raises yours. The strategy is cumulative: apply to ALL Priority-1 rows + the AIESEC fallback and your chance of landing at least ONE international win within 12 months is realistic (roughly 40–60% including AIESEC, ~15–25% for the fully-sponsored ones only). Priority: 1 = apply this cycle · 2 = opportunistic · 3 = later fork · X = don't waste time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Program</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Company / Org</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Country / Base</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Eligibility (incl. GPA reality)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>What's covered</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Next window for YOU</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>WHEN TO APPLY (aligned to your Apr-2027 start)</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>How to apply (steps)</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Official link</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Fit &amp; why (honest)</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>WHERE TO APPLY (direct links)</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>YOUR ODDS (honest, starting from zero)</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Fit &amp; why</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Applied on</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>Notes / Result</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>KPMG Global Internship Program (GIP)</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>KPMG</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>4 weeks abroad (US, UK, Singapore, Germany…)</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Big-4 sponsored internship abroad</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Must FIRST win a KPMG India internship — India is one of ~14 eligible countries. Undergrad/recent grad. No published GPA floor; selection is interview-based.</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>FULLY FUNDED by KPMG Global Mobility: flights, housing, stipend, visa support.</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>KPMG India internship portal ~Aug–Oct 2026 for the 2027 cycle; GIP internal application after your offer (late 2026–early 2027).</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>1) Apply for a KPMG India internship (careers site, non-audit tracks: advisory/marketing ops). 2) Once you have the offer, ask your recruiter about GIP nomination. 3) Complete the internal GIP application + interview.</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>kpmg.com/in → Careers → Internships</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>★★★ Your anchor bet. The ONLY Big-4 with a formal intern-abroad track open from India. No GPA screen at interview — sell Pack &amp; Pass ops + numbers.</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr"/>
-      <c r="N5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -686,63 +647,68 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Red Bull Basement</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Red Bull</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Global Final (city changes yearly)</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Student-founder program, sponsored travel</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Enrolled students 18+, any discipline, with a startup/idea. Zero academics in judging.</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>National winners flown to the Global Final — travel + stay covered by Red Bull.</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Applications typically open May–Sep 2026 — LIKELY OPEN NOW, check this week.</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>1) Go to redbullbasement.com. 2) Submit a 60-second pitch video of Pack &amp; Pass (or an AI-for-travel angle). 3) National selection → Global Final.</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>redbullbasement.com</t>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>KPMG Global Internship Program (GIP)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>KPMG</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>4 weeks abroad (US, UK, Singapore, Germany…)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Big-4 sponsored internship abroad (real internship)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Must FIRST win a KPMG India internship — India is one of ~14 GIP-eligible countries. Academic cutoff for KPMG India is usually 60%+; your 2.8/4.0 (~70%) clears it. Note: the flagship summer program targets penultimate-year students — as a final-year, target the year-round office internship postings (open to final-years/recent grads).</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>GIP leg FULLY FUNDED by KPMG Global Mobility: flights, housing, stipend, visa support. India internship pays ~₹30–80k/mo stipend.</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Apply AUG–NOV 2026 on the India portals for the Apr–Jul 2027 intake — this maps perfectly to your availability. GIP internal application comes after your India offer (~Dec 2026–Feb 2027).</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>1) Apply to KPMG India internship postings (advisory/markets/digital roles, not audit). 2) Also apply via LinkedIn/Unstop/Internshala where KPMG India posts. 3) After an offer, ask your recruiter about GIP nomination + internal application.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>kpmg.com/in/en/careers/students.html · kpmg.com/in/en/careers.html · linkedin.com/jobs (search 'KPMG India intern') · unstop.com · internshala.com (KPMG posts on all three)</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>★★★ Founder-first, zero GPA. You already have a live business — that's rare among applicants. Costs you one video.</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
+          <t>MEDIUM ~10–20% for the India internship (with referral + interview prep); LOW ~3–5% for the abroad GIP leg on top. Two-stage bet — the India internship alone is a win even if GIP doesn't land.</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>★★★ Anchor bet. Only Big-4 with a formal intern-abroad track open from India.</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr"/>
-      <c r="N6" s="6" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
+      <c r="O6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -750,63 +716,68 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>L'Oréal Brandstorm</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>L'Oréal</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Paris, France (finals)</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Global innovation/marketing competition → internship offers</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Ages 18–30, any discipline, team of 3 from India. India participates. No GPA anywhere in judging.</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>National winners fly to Paris finals — travel + stay fully sponsored. Winners frequently receive L'Oréal internships.</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>2027 edition opens ~Nov 2026; India registration closed ~3 Feb in the 2026 edition — expect similar.</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>1) Recruit 2 teammates now (marketing-minded juniors are fine). 2) Register at brandstorm.loreal.com when the 2027 edition opens. 3) Submit concept → national rounds → Paris.</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>brandstorm.loreal.com</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>★★★ Purpose-built for a marketer. Judged 100% on idea + pitch. A finals run is a resume headline that erases the GPA question.</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Red Bull Basement</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Global Final (city changes yearly)</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Student-founder COMPETITION (short event — do while studying)</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Enrolled students 18+, any discipline, with a startup/idea. Zero academics in judging. You must still be enrolled when you apply → apply THIS cycle, before you graduate.</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>National winners flown to the Global Final — travel + stay covered by Red Bull.</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Apply NOW: window typically runs Jul–Sep/Oct 2026; Global Final ~Dec 2026 (a few days — no clash with college). This is likely your ONLY eligible cycle.</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>1) Go to the Basement site. 2) Submit a 60-second pitch video of Pack &amp; Pass (or an AI-for-travel angle). 3) National selection → Global Final.</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>redbull.com/int-en/basement (redbullbasement.com redirects here)</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>LOW ~2–5% to win the national round — but the application costs you ONE hour and one video. Highest value-per-hour row on this sheet.</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>★★★ Founder-first, zero GPA. You already run a live business — rare among applicants.</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr"/>
-      <c r="N7" s="5" t="inlineStr"/>
+      <c r="N7" s="7" t="inlineStr"/>
+      <c r="O7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -814,63 +785,68 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>SUSI for Student Leaders</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>U.S. State Department</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>USA (5 weeks)</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Fully funded leadership institute</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Undergraduate, ages 18–25, Indian citizen, leadership record. No GPA floor — essays + leadership evidence. NOTE: you must still be an undergrad → the 2026–27 cycle is likely your LAST eligible one.</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>EVERYTHING: international flights, lodging, meals, full program costs.</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>U.S. Embassy New Delhi announces the cycle ~Oct 2026–Jan 2027. Watch for it monthly from Sep.</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>1) Follow in.usembassy.gov + U.S. Embassy India socials. 2) Email the Public Affairs Section (PAS) New Delhi asking for the SUSI 2027 call. 3) Apply with the Pack &amp; Pass founder story as your leadership evidence.</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>exchanges.state.gov/non-us/program/study-us-institutes-student-leaders</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>★★★ They select exactly your profile: young leader building something in his community. Last-chance timing makes this a must-apply.</t>
-        </is>
-      </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>L'Oréal Brandstorm</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>L'Oréal</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Paris, France (finals)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Marketing/innovation COMPETITION (event) → internship offers</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Ages 18–30, any discipline, team of 3 from India. India participates. No GPA anywhere in judging. Still eligible after graduation (18–30 age rule), so no timing panic.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>National winners fly to Paris finals — travel + stay fully sponsored. Winners frequently receive L'Oréal internships.</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>2027 edition: register ~NOV 2026 – early FEB 2027 (India deadline was 3 Feb in the 2026 edition). Finals mid-2027 — right after your graduation, timing is perfect.</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>1) Recruit 2 teammates now. 2) Register on the Brandstorm site when the 2027 edition opens (~Nov). 3) Submit concept → national rounds → Paris.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>brandstorm.loreal.com · unstop.com (L'Oréal India also lists it there)</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>LOW ~1–3% for Paris finals (thousands of Indian teams) — but MEDIUM odds of clearing early national rounds, and even that is strong resume proof.</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>★★★ Purpose-built for a marketer. Judged 100% on idea + pitch.</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr"/>
-      <c r="N8" s="6" t="inlineStr"/>
+      <c r="N8" s="5" t="inlineStr"/>
+      <c r="O8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -878,775 +854,905 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>SUSI for Student Leaders</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>U.S. State Department</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>USA (5 weeks)</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Fully funded leadership institute (short program)</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Undergraduate, ages 18–25, Indian citizen, leadership record. No GPA floor. ⚠ ELIGIBILITY FLAG: SUSI usually wants students with at least one semester REMAINING after the institute — you graduate Apr 2027 and institutes run summer 2027, so you may just miss the cutoff. Email PAS New Delhi FIRST to confirm before investing any time.</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>EVERYTHING: international flights, lodging, meals, full program costs.</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Watch SEP 2026 – JAN 2027 for the 2027 cycle announcement. Program runs summer 2027. Step zero (this month): the eligibility-confirmation email.</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>1) Email the Public Affairs Section, U.S. Embassy New Delhi asking for the SUSI 2027 call + whether a student graduating Apr 2027 is eligible. 2) Follow in.usembassy.gov + embassy socials. 3) If eligible, apply with the Pack &amp; Pass founder story.</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>exchanges.state.gov/non-us/program/study-us-institutes-student-leaders · in.usembassy.gov/education-culture (announcements)</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>LOW ~2–5% if eligible — and eligibility itself is uncertain for you. One email settles it; don't spend more than that until they answer.</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>★★★ profile fit, but timing is tight — this one is a conditional bet.</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="N9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Young Founders Programme</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Westerwelle Foundation</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Berlin, Germany (~1 week + alumni network)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Fully funded founder program</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Founders ~18–35 from emerging markets with a RUNNING business. Pack &amp; Pass qualifies today. No GPA.</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Fully funded founder program (short event — anytime)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Founders ~18–35 from emerging markets with a RUNNING business. Pack &amp; Pass qualifies today. No GPA. No student requirement — you stay eligible for years.</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Travel + accommodation in Berlin fully covered.</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Two cohorts/year (spring + autumn); autumn-cohort applications often run Jun–Aug — CHECK NOW.</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>1) westerwelle-foundation.com → Young Founders Programme. 2) Online application: pitch Pack &amp; Pass with real numbers (bookings, revenue, growth). 3) Interview round.</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>westerwelle-foundation.com</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>★★★ You qualify as-is. Also the best network row on this sheet: global founder alumni + follow-up conferences.</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Two cohorts/year. Spring-cohort applications historically open in JANUARY → apply JAN 2027. Also check the page THIS MONTH in case an autumn-2026 call is open. 1-week trip — fits around anything.</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>1) Open the program page and hit Apply if a call is open (form is on the page, bottom). 2) Pitch Pack &amp; Pass with real numbers: bookings, revenue, growth. 3) Interview round.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>westerwelle-foundation.com/programs/young-founders-program/ · vc4a.com (they post calls there too)</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM ~10–20% — the best odds of any sponsored row: you compete against a small pool of actual founders, not millions of students, and you have a real running business.</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>★★★ You qualify as-is TODAY. Also the best network row on this sheet.</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr"/>
-      <c r="N9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr"/>
+      <c r="O10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>P&amp;G CEO Challenge</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Procter &amp; Gamble</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Regional finals (Dubai/Singapore) → World final</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Business case competition, sponsored travel</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>University students, teams; India participates. No GPA in judging.</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Business case COMPETITION (event)</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>University students, teams; India participates. No GPA in judging. Apply while still enrolled → this cycle.</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Travel to regional + world finals covered; strong performers fast-tracked to P&amp;G internships.</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>India edition usually opens ~Sep–Dec 2026.</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>1) Register at pgcareers.com when the India edition opens. 2) Online case rounds → national → regional. 3) Use FMCG-style thinking practiced on Pack &amp; Pass campaigns.</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>pgcareers.com/ceo-challenge</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>★★☆ Very competitive but merit-only. Even a national-round finish is strong resume proof.</t>
-        </is>
-      </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>India edition usually opens SEP–DEC 2026; finals early-mid 2027 (short event, no clash). Likely your last eligible cycle as a student.</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>1) Register when the India edition opens. 2) Online case rounds → national → regional. 3) Use FMCG-style thinking practiced on Pack &amp; Pass campaigns.</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>pg-ceochallenge.com · pgcareers.com/CEO-Challenge</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>LOW ~2–5% to reach regionals. Treat as interview practice with a lottery ticket attached.</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>★★☆ Merit-only; even a national-round finish is resume proof.</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M10" s="6" t="inlineStr"/>
-      <c r="N10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="N11" s="7" t="inlineStr"/>
+      <c r="O11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Hult Prize</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Hult Prize Foundation</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Global Accelerator (residential) + Global Finals</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Social-impact startup competition</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>University students/teams. No GPA. Needs a social-impact frame.</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Social-impact startup COMPETITION (event + summer accelerator)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>University students/teams (enrolled at registration). No GPA. Needs a genuine social-impact frame.</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Global Accelerator is residential and covered for qualifying teams; US$1M for the winner.</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>OnCampus/OpenApplication rounds ~Sep–Dec 2026; nationals early 2027.</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>1) hultprize.org → register a team. 2) Frame Pack &amp; Pass as community/sustainable tourism for budget Indian travelers. 3) Campus round → nationals → accelerator.</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Register SEP–DEC 2026 (while still enrolled); nationals early 2027; accelerator summer 2027 — after your graduation, timing works.</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>1) Register a team on hultprize.org. 2) Frame Pack &amp; Pass as community/sustainable tourism for budget Indian travelers. 3) Campus round → nationals → accelerator.</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>hultprize.org</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>★★☆ Works only if the social-impact angle is genuine — community-based tourism / accessible travel documentation is a credible frame.</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>LOW–MEDIUM ~5–10% to win a campus/national round (depends how contested your campus is); LOW for the accelerator.</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>★★☆ Only if the social-impact angle is genuine — accessible travel documentation is a credible frame.</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr"/>
-      <c r="N11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr"/>
+      <c r="O12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>UFLL / L.E.A.P (→ UFLP internship)</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Unilever (HUL)</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>India → global final (travel covered historically)</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>Competition → flagship internship pathway</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Students in India; team-based. No GPA in judging (assessment-centre based).</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Global-final travel covered in past editions; winners get fast-track to HUL internships (ULIP).</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>India campus season ~Jan–Mar 2027 — verify current format on Unilever India careers.</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>1) Watch careers.unilever.com/india from Dec 2026. 2) Register for the current competition (name varies by year). 3) Assessment centre → final.</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>careers.unilever.com/india</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>★★☆ Format changes yearly — confirm before investing time. Brand value is top-tier for a marketer.</t>
-        </is>
-      </c>
-      <c r="L12" s="6" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Students in India; team-based. No GPA in judging (assessment-centre based). Format and name change yearly — verify before investing time.</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Global-final travel covered in past editions; winners fast-track to HUL internships.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>India campus season JAN–MAR 2027; any internship prize lands summer 2027 → fits your April availability.</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>1) Watch Unilever India careers from Dec 2026. 2) Register for the current competition (check Unstop too — HUL runs its India challenges there). 3) Assessment centre → final.</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>careers.unilever.com/india · unstop.com (search 'HUL' / 'Unilever')</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>LOW ~2–5%. Brand value is top-tier for a marketer, so worth one application cycle.</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>★★☆ Verify current format first.</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M12" s="6" t="inlineStr"/>
-      <c r="N12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="N13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>UNICEF Internship (Comms/Digital roles)</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>UNICEF</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Various country offices + HQ</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>UN body, paid internship</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Enrolled students OR within 2 years of graduation. They ask for academic records and 'excellent performance' — your 2.8 is a real handicap here; offset with portfolio + two strong references.</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>UN body, paid REAL internship</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Enrolled students OR within 2 years of graduation → you stay eligible until Apr 2029. They ask for academic records; your 2.8 is a real handicap — offset with portfolio + references.</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Monthly stipend + one-time lump sum toward visa/travel.</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Rolling — postings appear year-round. Set a monthly check reminder.</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>1) unicef.org/careers → search 'internship'. 2) Filter for communication/digital/marketing postings. 3) Apply per-posting with portfolio links up front.</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>unicef.org/careers</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>★★☆ Low cost to try since it's rolling. Target comms/digital roles where portfolio outweighs transcripts.</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Start applying JAN–FEB 2027 for Apr-2027+ starts (postings run 1–3 months ahead). Then keep a monthly check through 2027–28 — your eligibility window is long.</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>1) Go to the UNICEF jobs portal, filter category = Internship. 2) Apply only to communication/digital/marketing postings. 3) Portfolio links in the first line of every cover letter.</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>jobs.unicef.org (filter: Internship)</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>LOW ~3–8% per posting — but it's rolling, so repeated applications compound. Budget 1 application/month, not hope.</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>★★☆ Target roles where the work sample outweighs the transcript.</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr"/>
-      <c r="N13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="N14" s="5" t="inlineStr"/>
+      <c r="O14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>ILO Internship</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Int'l Labour Organization (UN)</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>Geneva + field offices</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>UN body, stipended internship</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Grad/postgrad students or recently graduated (~within 1 year). For you: usable May 2027–Apr 2028, right after graduation. GPA not the filter — relevance is.</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>UN body, stipended REAL internship</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Grad/postgrad students or recently graduated (~within 1 year) → your usable window is MAY 2027 – APR 2028, right after graduation. GPA not the filter — relevance is.</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Stipend (~CHF 1,850–2,340/mo in Geneva) if not otherwise funded. Travel NOT covered.</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>Internship roster opens ~2×/year — check Jan + Jul 2027.</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>1) ilo.org/careers → Internships. 2) Apply to the roster in the window right after you graduate. 3) Pitch the youth-employment/entrepreneurship angle with Pack &amp; Pass.</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>ilo.org → Careers → Internships</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="inlineStr">
-        <is>
-          <t>★☆☆ Partial funding + grad-level tilt. Park until mid-2027.</t>
-        </is>
-      </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Roster opens ~2×/year — apply in the JAN 2027 and JUL 2027 windows for placements after your April graduation.</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>1) ILO jobs portal → Internship roster. 2) Apply in-window with the youth-employment/entrepreneurship angle (Pack &amp; Pass). 3) Named-official follow-up if shortlisted.</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>jobs.ilo.org (search 'internship roster')</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>LOW ~3–5%, and travel is on you. A year-2 card, not a year-1 priority.</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>★☆☆ Partial funding; park until 2027.</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr"/>
-      <c r="N14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="N15" s="7" t="inlineStr"/>
+      <c r="O15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>WTO Internship</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>World Trade Organization</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Geneva, Switzerland</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>UN-style body, paid internship</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>POSTGRADUATE students only → this is a Fork-A (MBA/Masters years 3–4) card, not a now card.</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>CHF 60/day allowance + travel expenses covered.</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Only if you do a Masters/MBA (2028+).</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>1) Park this. 2) If Fork A happens, apply via wto.org internship page during your Masters.</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>wto.org → internships</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>★☆☆ Good money + brand, but locked behind postgrad status.</t>
-        </is>
-      </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Paid internship — POSTGRAD only</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Postgraduate students only → a Fork-A (Masters/MBA, years 3–4) card, not a now card.</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>CHF 60/day allowance + travel covered.</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Only if you do a Masters/MBA → 2028 at the earliest. Nothing to do before then.</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>1) Park it. 2) If Fork A happens, apply via the WTO internship page during your Masters.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>wto.org/english/thewto_e/vacan_e/intern_e.htm</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>N/A today (0% — eligibility gate). Decent odds later IF you're a postgrad.</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>★☆☆ Locked behind postgrad status.</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr"/>
-      <c r="N15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="N16" s="5" t="inlineStr"/>
+      <c r="O16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>OECD Internship</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>OECD</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Paris, France</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Paid internship (€~1,000/mo)</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>SKIP: primarily for nationals of OECD member countries — India is not a member. Travel also not covered.</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>€1,000/mo, no travel.</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>— (don't apply)</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>Don't spend time here; the nationality rule kills the odds.</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>oecd.org/careers</t>
-        </is>
-      </c>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
-          <t>✗ Included so you don't waste a week on it later.</t>
-        </is>
-      </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>oecd.org/careers/internship-programme</t>
+        </is>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>~0% — nationality gate.</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>✗ Kept so you don't waste a week on it later.</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="M16" s="6" t="inlineStr"/>
-      <c r="N16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="N17" s="7" t="inlineStr"/>
+      <c r="O17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Mitacs Globalink</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Mitacs (Canada)</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Funded research internship</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>SKIP: hard GPA floor (~8.0/10 ≈ 3.2+/4.0) and research/STEM-heavy. Your 2.8 is below the cutoff — application would be auto-filtered.</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>SKIP: hard GPA floor (~8.0/10 ≈ 3.2+/4.0) and research/STEM-heavy. Your 2.8 is below the automated cutoff.</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Fully funded (when eligible).</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>— (don't apply)</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Don't apply; the GPA filter is automated.</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>mitacs.ca</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>✗ Honest skip — this is the type of program the GPA actually blocks.</t>
-        </is>
-      </c>
-      <c r="L17" s="5" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>mitacs.ca/our-programs/globalink-research-internship</t>
+        </is>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>~0% — automated GPA filter.</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>✗ The kind of program the GPA actually blocks.</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="M17" s="5" t="inlineStr"/>
-      <c r="N17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="N18" s="5" t="inlineStr"/>
+      <c r="O18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>DAAD WISE</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>DAAD (Germany)</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>Funded research internship</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>SKIP: STEM/engineering students only.</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>Scholarship + travel (when eligible).</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>— (don't apply)</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>Not your field — skip.</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
-        <is>
-          <t>daad.in</t>
-        </is>
-      </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>daad.in (WISE page)</t>
+        </is>
+      </c>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>0% — field gate.</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
         <is>
           <t>✗ Listed only to close the question.</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="M19" s="7" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="M18" s="6" t="inlineStr"/>
-      <c r="N18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="N19" s="7" t="inlineStr"/>
+      <c r="O19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>AIESEC Global Talent (Marketing)</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>AIESEC</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>SE Asia / Europe / LatAm</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Paid work placement abroad (NOT sponsored travel)</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Paid work placement abroad — REAL internship (NOT sponsored travel)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>Ages 18–30. No GPA. Honest catch: AIESEC charges a program fee (~₹35–45k) and you fund your own flight; the internship salary covers living costs abroad.</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Salary covers living; fee + flights are on you → 'earn-while-abroad', not 'fully funded'.</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>Rolling — placements posted continuously.</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>1) aiesec.org → Global Talent → marketing roles. 2) Apply to specific placements. 3) Interview with the host company.</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>aiesec.org</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>★★☆ The realistic fallback if the sponsored bets don't land — a paid marketing job abroad on your CV by late 2027.</t>
-        </is>
-      </c>
-      <c r="L19" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Create your profile DEC 2026; apply to placements JAN–FEB 2027 — matching + visa takes 2–3 months, landing you abroad right around APR 2027.</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>1) Sign up on aiesec.org. 2) Browse Global Talent marketing placements and apply to specific ones. 3) Interview with the host company. 4) Local AIESEC chapter handles logistics.</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>aiesec.org/global-talent (live placements listed on the page)</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>HIGH ~40–60% — this is a placement marketplace, not a scholarship. If you interview decently and pay the fee, you get placed. Your one near-certain route abroad.</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>★★☆ The safety net: a paid marketing job abroad on your CV by mid-2027 even if every sponsored bet misses.</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M19" s="5" t="inlineStr"/>
-      <c r="N19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="N20" s="5" t="inlineStr"/>
+      <c r="O20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>EY / Deloitte / PwC India internships</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>EY, Deloitte, PwC</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>India (abroad = later)</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>Big-4 brand internships (no intern-abroad track from India)</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>Honest note: unlike KPMG, none of these three runs a formal India→abroad INTERN program. Their global mobility/secondments come 1–3 years AFTER you join full-time.</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Honest note: unlike KPMG, none of these three runs a formal India→abroad INTERN program. Their global mobility/secondments come 1–3 years AFTER joining full-time. Academic cutoffs ~60% — you clear them.</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>Standard India internship stipend only.</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>Portals open ~Aug–Nov 2026 alongside your existing India tracker.</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>1) Apply via each careers portal (already on your India list). 2) Treat as brand-building + a 2-year route to sponsored mobility as an employee.</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>ey.com/in · deloitte.com/in · pwc.in</t>
-        </is>
-      </c>
-      <c r="K20" s="6" t="inlineStr">
-        <is>
-          <t>★☆☆ For the abroad goal specifically, KPMG is the play; these three are brand plays.</t>
-        </is>
-      </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Apply AUG–NOV 2026 for the 2027 intake (Apr 2027+ start fits you). Same season as KPMG — batch these applications together.</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>1) Apply on each India careers portal + LinkedIn. 2) Treat as brand-building + a 2-year route to sponsored mobility as an employee.</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>careers.ey.com + ey.com/en_in/careers · deloitte.com/in/en/careers.html · pwc.in/careers.html</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM ~10–15% each with referrals + prep (same interview prep as KPMG reuses here).</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>★☆☆ For the abroad goal KPMG is the play; these are brand plays.</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="M20" s="6" t="inlineStr"/>
-      <c r="N20" s="6" t="inlineStr"/>
+      <c r="N21" s="7" t="inlineStr"/>
+      <c r="O21" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A1:N1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A3:O3"/>
+    <mergeCell ref="A2:O2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="L5:L20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M6:M21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,Researching,Preparing,Applied,Interview,Accepted,Rejected,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1676,17 +1782,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>Rule / Move</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>Exactly what to do</t>
         </is>
@@ -1710,17 +1816,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Build the 4 reusable assets ONCE (this month, Jul 2026)</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>(a) One-page founder-first CV (structure on PLAN sheet). (b) 90-second pitch video of Pack &amp; Pass — reused for Red Bull Basement, Westerwelle, Brandstorm. (c) A 3-page Pack &amp; Pass case-study PDF with REAL numbers: bookings handled, revenue, Instagram growth, one campaign's results. (d) LinkedIn profile that matches all of it. Every application on the tracker draws from these four.</t>
         </is>
@@ -1744,17 +1850,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Lead every application with proof, not adjectives</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>First sentence of every essay/cover letter = a concrete result: 'I run Pack &amp; Pass, a travel agency that has handled X bookings and ₹Y in revenue for South Indian budget travelers.' Interviewers remember one number better than ten adjectives.</t>
         </is>
@@ -1778,17 +1884,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>KPMG GIP angle</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>The India internship interview is the real gate. Prep 3 stories from Pack &amp; Pass: (1) handling a client crisis (visa rejection/last-minute change), (2) a campaign that produced measurable bookings, (3) unit economics of a trip package. That's business acumen no classroom candidate can match. THEN ask the recruiter about GIP — knowing it exists signals ambition.</t>
         </is>
@@ -1812,17 +1918,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>SUSI / embassy programs angle</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>They select for leadership + community impact, not marks. Frame Pack &amp; Pass as making travel/documentation accessible to first-time South Indian travelers — a community story, told with 2–3 named examples of people you helped.</t>
         </is>
@@ -1846,17 +1952,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>UNICEF / UN bodies angle</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>The one place transcripts get seen. Compensate: portfolio links in the FIRST line of the cover letter, referee who can vouch for output, and apply only to comms/digital postings where the work sample matters most. Accept lower odds; it's rolling so each attempt costs little.</t>
         </is>
@@ -1875,22 +1981,22 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>From the tracker: Jul–Aug = Red Bull Basement + Westerwelle check + assets. Aug–Oct = KPMG India (+ EY/Deloitte/PwC brand plays). Sep–Dec = P&amp;G, Hult, SUSI watch. Nov–Feb = Brandstorm 2027. Rolling = UNICEF monthly check. Update the Status column weekly — treat it like a sales pipeline.</t>
+          <t>From the tracker: Jul–Aug = Red Bull Basement + Westerwelle check + assets. Aug–Nov = KPMG India (+ EY/Deloitte/PwC brand plays). Sep–Dec = P&amp;G, Hult, SUSI watch. Nov–Feb = Brandstorm 2027. Dec–Feb = AIESEC profile + applications. Rolling = UNICEF monthly check. Update the Status column weekly — treat it like a sales pipeline.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>After every rejection</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Log it in Notes, ask for feedback once (politely, many programs answer), and recycle the material into the next application. The assets compound; the rejections don't.</t>
         </is>
@@ -1919,24 +2025,24 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>THE REST OF THE PDF BRIEF — CONDENSED (details live in CAREER_GROWTH_CALENDAR.md in this repo)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Brief item</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>The answer in short</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>When</t>
         </is>
@@ -1960,17 +2066,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>BIG ROCK 2 — A tech-company internship (India)</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Already the spine of your existing calendar: apply Aug–Dec 2026 for the Apr–Jul 2027 cycle. KPMG India now joins that list because it unlocks the GIP abroad track.</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Aug–Dec 2026</t>
         </is>
@@ -1994,17 +2100,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>BIG ROCK 4 — Certifications as seasoning, not the meal</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Google Ads + GA4 (Skillshop, free), Meta Blueprint, HubSpot content — already scheduled Dec 2026–Jan 2027 in your calendar. They pass HR filters; the campaign case study wins the interview.</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Dec 2026–Jan 2027</t>
         </is>
@@ -2028,17 +2134,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>LINKEDIN — headline</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>'Founder, Pack &amp; Pass Travels | Digital Marketing | I build &amp; ship — campaigns, funnels, travel products'. About section: 3 short paragraphs — what you run, what you've shipped (numbers), what you're looking for. No GPA, no 'aspiring'.</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>this week</t>
         </is>
@@ -2062,17 +2168,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>RESUME — structure that buries a 2.8</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Order: Name/contact → 2-line summary (founder + marketer) → EXPERIENCE (Pack &amp; Pass first, with 3 numeric bullets) → Projects/Campaigns → Skills &amp; Certifications → Education LAST, one line, degree + college + year, NO GPA. If a portal forces GPA into a field, give it there — never on the document.</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>this week</t>
         </is>
@@ -2096,17 +2202,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>FORK B (no MBA — build + compound)</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Yrs 1–2: marketing job + Pack &amp; Pass on the side. Yr 3: senior/freelance premium work, Pack &amp; Pass systematized with AI tooling. Yr 4: full one-person business (agency-of-one: marketing services + travel products). Network and shipped work replace the credential.</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>default path</t>
         </is>

</xml_diff>